<commit_message>
prefix nama tabel sinta
</commit_message>
<xml_diff>
--- a/scripts/output/merged_data_6165083.xlsx
+++ b/scripts/output/merged_data_6165083.xlsx
@@ -12,12 +12,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCOPUS_YEARLY_STATS" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCHOLAR_PUBLICATIONS" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCHOLAR_YEARLY_STATS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GARUDA" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOOKS" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERVICES" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERVICE_YEARLY" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESEARCHES" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESEARCH_YEARLY" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GARUDA_PUBLICATIONS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GARUDA_YEARLY_STATS" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOOKS" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERVICES" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERVICE_YEARLY" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESEARCHES" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESEARCH_YEARLY" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -539,89 +540,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>judul</t>
+          <t>tahun</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>leader</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>skema</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>personils</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>tahun</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>dana</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>source</t>
+          <t>jumlah</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Pengembangan Modul Matematika Untuk Siswa    Kelas 3 Sekolah Dasar Negeri Wujil 01 Bergas</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Mochamad Rizqi Adhi Pratama</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Penelitian Kompetitif Nasional ( PDP/Dosen Pemula )</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Personils : Nur Intan Rochmawati ;</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
+      <c r="A2" t="n">
         <v>2019</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Rp. 20.000.000</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>BIMA SOURCE</t>
-        </is>
+      <c r="B2" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -630,6 +569,102 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>judul</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>leader</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>skema</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>personils</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tahun</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>dana</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Pengembangan Modul Matematika Untuk Siswa    Kelas 3 Sekolah Dasar Negeri Wujil 01 Bergas</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mochamad Rizqi Adhi Pratama</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Penelitian Kompetitif Nasional ( PDP/Dosen Pemula )</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Personils : Nur Intan Rochmawati ;</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2019</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Rp. 20.000.000</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>BIMA SOURCE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -853,22 +888,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OPTIMALISASI PENGEMBANGAN KOGNITIF ANAK TK A MENGGUNAKAN ALAT PERMAINAN EDUKATIF MATCH COLOUR FINE MOTOR BALL DI TK BUMITAMA</t>
+          <t>Comparative Analysis of Facilities and Infrastructure in Urban and Rural Early Childhood Education Centers (TPA) in Indonesia Toward Achieving Quality Early Childhood Education …</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'OPTIMALISASI PENGEMBANGAN KOGNITIF ANAK TK A MENGGUNAKAN ALAT PERMAINAN EDUKATIF MATCH COLOUR FINE MOTOR BALL DI TK BUMITAMA'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Comparative Analysis of Facilities and Infrastructure in Urban and Rural Early Childhood Education Centers (TPA) in Indonesia Toward Achieving Quality Early Childhood Education …'</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>RE Astuti, NI Rochmawati, HH Taulany, SSI Prahesti</t>
+          <t>IMP Pratiwi, IK Nisa, NI Rochmawati</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Pendas: Jurnal Ilmiah Pendidikan Dasar 11 (01), 45-58, 2026</t>
+          <t>Journal of Educational Innovation and Research 2 (1), 549-553, 2026</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -884,22 +919,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MANAJEMEN PEMBIAYAAN PENDIDIKAN DALAM DINAMIKA KEBIJAKAN PENDIDIKAN MENENGAH</t>
+          <t>EVALUATING TV SEKOLAH AS AN EVIDENCE-BASED TOOL FOR PAUD HI PROGRAM EVALUATION AND DIGITAL CHILD PORTFOLIOS IN KINDERGARTEN SETTINGS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'MANAJEMEN PEMBIAYAAN PENDIDIKAN DALAM DINAMIKA KEBIJAKAN PENDIDIKAN MENENGAH'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'EVALUATING TV SEKOLAH AS AN EVIDENCE-BASED TOOL FOR PAUD HI PROGRAM EVALUATION AND DIGITAL CHILD PORTFOLIOS IN KINDERGARTEN SETTINGS'</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>D Hardanti, AJ Mahardhani, LF Adipura, NI Rochmawati, S Septiani</t>
+          <t>NI Rochmawati, W Pudjaningsih, A Pratama, DD Fyanthusany</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>EDUPEDIA 10 (1), 81-90, 2026</t>
+          <t>Pendas: Jurnal Ilmiah Pendidikan Dasar 11 (01), 240-252, 2026</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -915,22 +950,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ADAPTIVE INSTRUCTIONAL LEADERSHIP IN RESOURCE-CONSTRAINED KINDERGARTENS: A QUALITATIVE STUDY OF PRINCIPALS’STRATEGIES</t>
+          <t>LEADING DEEP LEARNING IN PRIMARY EDUCATION: HOW SCHOOL PRINCIPALS LEVERAGE TEACHER LEARNING COMMUNITIES TO ENHANCE EDUCATIONAL QUALITY</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'ADAPTIVE INSTRUCTIONAL LEADERSHIP IN RESOURCE-CONSTRAINED KINDERGARTENS: A QUALITATIVE STUDY OF PRINCIPALS’STRATEGIES'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'LEADING DEEP LEARNING IN PRIMARY EDUCATION: HOW SCHOOL PRINCIPALS LEVERAGE TEACHER LEARNING COMMUNITIES TO ENHANCE EDUCATIONAL QUALITY'</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>P Darwanti, NI Rochmawati</t>
+          <t>B Nurasih, NI Rochmawati</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>El Midad 18 (1), 40-49, 2026</t>
+          <t>El Midad 18 (1), 61-71, 2026</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -946,29 +981,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IMPLEMENTASI KEGIATAN SENAM IRAMA DALAM MENGEMBANGKAN KEMAMPUAUN MOTORIK KASAR ANAK USIA 5-6 TAHUN DI TK ISLAM MASJID AL FALAQ</t>
+          <t>Transparansi dan Akuntabilitas Pengelolaan Dana Bantuan Operasional Sekolah (BOS) di Indonesia: Systematic Literature Review</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'IMPLEMENTASI KEGIATAN SENAM IRAMA DALAM MENGEMBANGKAN KEMAMPUAUN MOTORIK KASAR ANAK USIA 5-6 TAHUN DI TK ISLAM MASJID AL FALAQ'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Transparansi dan Akuntabilitas Pengelolaan Dana Bantuan Operasional Sekolah (BOS) di Indonesia: Systematic Literature Review'</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>AJ Ratnaningsih, W Pudjaningsih, S Fauziah, NI Rochmawati</t>
+          <t>DB Sulistyo, DMK Nufus, A Hidayah, NI Rochmawati, S Septiani</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Didaktik: Jurnal Ilmiah PGSD STKIP Subang 12 (01), 49-60, 2026</t>
+          <t>Jurnal Ilmiah Multidisiplin Mahasiswa dan Akademisi 1 (6), 90-105, 2026</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>2026</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -977,22 +1012,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Strategi Manajemen Pembiayaan Pendidikan Dalam Meningkatkan Mutu Lulusan</t>
+          <t>OPTIMALISASI PENGEMBANGAN KOGNITIF ANAK TK A MENGGUNAKAN ALAT PERMAINAN EDUKATIF MATCH COLOUR FINE MOTOR BALL DI TK BUMITAMA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Strategi Manajemen Pembiayaan Pendidikan Dalam Meningkatkan Mutu Lulusan'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'OPTIMALISASI PENGEMBANGAN KOGNITIF ANAK TK A MENGGUNAKAN ALAT PERMAINAN EDUKATIF MATCH COLOUR FINE MOTOR BALL DI TK BUMITAMA'</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>N Safira, A Rismaida, WT Setyobudi, NI Rochmawati, S Septiani</t>
+          <t>RE Astuti, NI Rochmawati, HH Taulany, SSI Prahesti</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Jurnal Ilmiah Multidisiplin Mahasiswa dan Akademisi 1 (6), 131-147, 2026</t>
+          <t>Pendas: Jurnal Ilmiah Pendidikan Dasar 11 (01), 45-58, 2026</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -1008,22 +1043,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IMPLEMENTASI PENGEMBANGAN ANAK USIA DINI HOLISTIK INTEGRATIF SEBAGAI STRATEGI DALAM MEMPERKUAT LAYANAN PERLINDUNGAN DAN PEMENUHAN HAK ANAK DI TK ISRIYATI SUGITO</t>
+          <t>MANAJEMEN PEMBIAYAAN PENDIDIKAN DALAM DINAMIKA KEBIJAKAN PENDIDIKAN MENENGAH</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'IMPLEMENTASI PENGEMBANGAN ANAK USIA DINI HOLISTIK INTEGRATIF SEBAGAI STRATEGI DALAM MEMPERKUAT LAYANAN PERLINDUNGAN DAN PEMENUHAN HAK ANAK DI TK ISRIYATI SUGITO'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'MANAJEMEN PEMBIAYAAN PENDIDIKAN DALAM DINAMIKA KEBIJAKAN PENDIDIKAN MENENGAH'</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>S Nasekah, NI Rochmawati, H Taulany, NK Dewi</t>
+          <t>D Hardanti, AJ Mahardhani, LF Adipura, NI Rochmawati, S Septiani</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Didaktik: Jurnal Ilmiah PGSD STKIP Subang 12 (01), 65-75, 2026</t>
+          <t>EDUPEDIA 10 (1), 81-90, 2026</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -1039,22 +1074,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Comparative Analysis of Facilities and Infrastructure in Urban and Rural Early Childhood Education Centers (TPA) in Indonesia Toward Achieving Quality Early Childhood Education …</t>
+          <t>ADAPTIVE INSTRUCTIONAL LEADERSHIP IN RESOURCE-CONSTRAINED KINDERGARTENS: A QUALITATIVE STUDY OF PRINCIPALS’STRATEGIES</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Comparative Analysis of Facilities and Infrastructure in Urban and Rural Early Childhood Education Centers (TPA) in Indonesia Toward Achieving Quality Early Childhood Education …'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'ADAPTIVE INSTRUCTIONAL LEADERSHIP IN RESOURCE-CONSTRAINED KINDERGARTENS: A QUALITATIVE STUDY OF PRINCIPALS’STRATEGIES'</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>IMP Pratiwi, IK Nisa, NI Rochmawati</t>
+          <t>P Darwanti, NI Rochmawati</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Journal of Educational Innovation and Research 2 (1), 549-553, 2026</t>
+          <t>El Midad 18 (1), 40-49, 2026</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -1070,22 +1105,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EVALUATING TV SEKOLAH AS AN EVIDENCE-BASED TOOL FOR PAUD HI PROGRAM EVALUATION AND DIGITAL CHILD PORTFOLIOS IN KINDERGARTEN SETTINGS</t>
+          <t>Strategi Manajemen Pembiayaan Pendidikan Dalam Meningkatkan Mutu Lulusan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'EVALUATING TV SEKOLAH AS AN EVIDENCE-BASED TOOL FOR PAUD HI PROGRAM EVALUATION AND DIGITAL CHILD PORTFOLIOS IN KINDERGARTEN SETTINGS'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Strategi Manajemen Pembiayaan Pendidikan Dalam Meningkatkan Mutu Lulusan'</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NI Rochmawati, W Pudjaningsih, A Pratama, DD Fyanthusany</t>
+          <t>N Safira, A Rismaida, WT Setyobudi, NI Rochmawati, S Septiani</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Pendas: Jurnal Ilmiah Pendidikan Dasar 11 (01), 240-252, 2026</t>
+          <t>Jurnal Ilmiah Multidisiplin Mahasiswa dan Akademisi 1 (6), 131-147, 2026</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1101,22 +1136,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LEADING DEEP LEARNING IN PRIMARY EDUCATION: HOW SCHOOL PRINCIPALS LEVERAGE TEACHER LEARNING COMMUNITIES TO ENHANCE EDUCATIONAL QUALITY</t>
+          <t>IMPLEMENTASI KEGIATAN SENAM IRAMA DALAM MENGEMBANGKAN KEMAMPUAUN MOTORIK KASAR ANAK USIA 5-6 TAHUN DI TK ISLAM MASJID AL FALAQ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'LEADING DEEP LEARNING IN PRIMARY EDUCATION: HOW SCHOOL PRINCIPALS LEVERAGE TEACHER LEARNING COMMUNITIES TO ENHANCE EDUCATIONAL QUALITY'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'IMPLEMENTASI KEGIATAN SENAM IRAMA DALAM MENGEMBANGKAN KEMAMPUAUN MOTORIK KASAR ANAK USIA 5-6 TAHUN DI TK ISLAM MASJID AL FALAQ'</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>B Nurasih, NI Rochmawati</t>
+          <t>AJ Ratnaningsih, W Pudjaningsih, S Fauziah, NI Rochmawati</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>El Midad 18 (1), 61-71, 2026</t>
+          <t>Didaktik: Jurnal Ilmiah PGSD STKIP Subang 12 (01), 49-60, 2026</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -1132,29 +1167,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Transparansi dan Akuntabilitas Pengelolaan Dana Bantuan Operasional Sekolah (BOS) di Indonesia: Systematic Literature Review</t>
+          <t>IMPLEMENTASI PENGEMBANGAN ANAK USIA DINI HOLISTIK INTEGRATIF SEBAGAI STRATEGI DALAM MEMPERKUAT LAYANAN PERLINDUNGAN DAN PEMENUHAN HAK ANAK DI TK ISRIYATI SUGITO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Transparansi dan Akuntabilitas Pengelolaan Dana Bantuan Operasional Sekolah (BOS) di Indonesia: Systematic Literature Review'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'IMPLEMENTASI PENGEMBANGAN ANAK USIA DINI HOLISTIK INTEGRATIF SEBAGAI STRATEGI DALAM MEMPERKUAT LAYANAN PERLINDUNGAN DAN PEMENUHAN HAK ANAK DI TK ISRIYATI SUGITO'</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>DB Sulistyo, DMK Nufus, A Hidayah, NI Rochmawati, S Septiani</t>
+          <t>S Nasekah, NI Rochmawati, H Taulany, NK Dewi</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Jurnal Ilmiah Multidisiplin Mahasiswa dan Akademisi 1 (6), 90-105, 2026</t>
+          <t>Didaktik: Jurnal Ilmiah PGSD STKIP Subang 12 (01), 65-75, 2026</t>
         </is>
       </c>
       <c r="F11" t="n">
         <v>2026</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1298,20 +1333,546 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>judul</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>url_artikel</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>publisher</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>url_journal</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>author_order</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>authors</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>tahun</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>doi</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>accreditation</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Transparansi dan Akuntabilitas Pengelolaan Dana Bantuan Operasional Sekolah (BOS) di Indonesia: Systematic Literature Review</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/documents/detail/5860899</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Prodi PGSD Unsultra</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Jurnal Ilmiah Multidisiplin Mahasiswa dan Akademisi Vol. 1 No. 6 (2026): Edisi Januari 202690 - 105</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/journal/view/42089</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>4 of 5</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Dian Bayu Sulistyo; Dyah Mutiara Khayatun Nufus; Anwirotul Hidayah; Nur Intan Rochmawati; Sisca Septiani</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>10.64690/intelektual.v1i6.586</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Strategi Manajemen Pembiayaan Pendidikan Dalam Meningkatkan Mutu Lulusan</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/documents/detail/5860905</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Prodi PGSD Unsultra</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Jurnal Ilmiah Multidisiplin Mahasiswa dan Akademisi Vol. 1 No. 6 (2026): Edisi Januari 2026131 - 147</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/journal/view/42089</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>4 of 5</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Najwa Safira; Anik Rismaida; Wahyu Tri Setyobudi; Nur Intan Rochmawati; Sisca Septiani</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>10.64690/intelektual.v1i6.611</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pendampingan Guru dan Komite SMK dalam Penguatan Pembelajaran Mendalam dan Karakter Siswa Berbasis Kurikulum Merdeka: Pengabdian</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/documents/detail/5750830</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Lembaga Penelitian dan Pengabdian Masyarakat</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Jurnal Pengabdian Masyarakat dan Riset Pendidikan Vol. 4 No. 2 (2025): Jurnal Pengabdian Masyarakat dan Riset Pendidikan Volume 4 Nomor 2 (October 20210029-10039</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/journal/view/34321</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2 of 5</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Lisa Virdinarti Putra; Nur Intan Rochmawati; Wiwik Pudjaningsih; Aulia Cahyaning Tyas; Bagas Prakosa</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>10.31004/jerkin.v4i2.3467</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Sinta 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Pendampingan Pemanfaatan Media TV Sekolah Sebagai Implementasi Pembelajaran Kontekstual Upaya Mendukung Sekolah Ramah Anak (SRA)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/documents/detail/6047286</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Universitas Ngudi Waluyo</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Multimatrix Vol. 4 No. 1 (2022): Kemajuan Teknologi Informatika Pada Era Dunia Digital</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/journal/view/45258</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2 of 3</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Arista Candra Irawati; Nur Intan Rochmawati; Abdul Rohman</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PENDIDIKAN BAGI ANAK USIA DINI ANAK IMIGRAN KORBAN PERANG DALAM MASA NEW NORMAL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/documents/detail/2715804</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Badan Perencanaan, Penelitian Dan Pengembangan Daerah, Kabupaten Semarang</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Media Informasi Penelitian Kabupaten Semarang Vol. 2 No. 2 (2020): Desember: Media Informasi Penelitian Kabupaten Semarang191-201</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/journal/view/24728</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1 of 2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Nur Intan Rochmawati; Adhi Budi Susilo</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>2020</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>10.55606/sinov.v3i2.83</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Pemanfaatan Aplikasi Zoom dan Google Meet Untuk Pembelajaran Daring di TK Pembina ABA 54 dan KB Ã¢â¬ËAisyiyah 18 Semarang</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/documents/detail/6047267</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Universitas Ngudi Waluyo</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Multimatrix Vol. 2 No. 2 (2020): Inovasi Teknologi Pada Masa Pademik Covid-19</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/journal/view/45258</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2 of 2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Abdul Rohman; Nur Intan Rochmawati</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>2020</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>POLA ASUH PERMISIF TERHADAP PENGEMBANGAN ARTIKULASI BAHASA ANAK USIA 4-5 TAHUN</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/documents/detail/1679386</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Jurusan PG-PAUD Universitas Halu Oleo</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Jurnal Smart PAUD Vol 2, No 1: Januari 201931-36</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/journal/view/12144</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1 of 1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>2019</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>10.36709/jspaud.v2i1.5917</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Sinta 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DONGENG SEBELUM TIDUR DALAM MENINGKATKAN KECERDASAN EMOSIONAL ANAK 4-5 TAHUN</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/documents/detail/1817360</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Universitas Ngudi Waluyo</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Indonesian Journal of Early Childhood: Jurnal Dunia Anak Usia Dini Vol 1, No 2 (2019)54-61</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/journal/view/19157</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1 of 1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>2019</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>10.35473/ijec.v1i2.357</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Sinta 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PENGOLAHAN SAMPAH PLASTIK MELALUI PEMANFAATAN KERAJINAN TANGAN PENDUKUNG BUDAYA SEHAT DESA SIDOMULYO KECAMATAN UNGARAN TIMUR</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/documents/detail/1106984</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Universitas Wahid Hasyim Semarang</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ABDIMAS UNWAHAS Vol 4, No 2 (2019)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/journal/view/16654</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2 of 3</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Adhi Budi Susilo; Nur Intan Rochmawati; Khifni Kafa Rufaida</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>2019</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>10.31942/abd.v4i2.3008</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Sinta 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DONGENG SEBELUM TIDUR DALAM MENINGKATKAN KECERDASAN EMOSIONAL ANAK 4-5 TAHUN</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/documents/detail/3483462</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Universitas Ngudi Waluyo</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Indonesian Journal of Early Childhood: Jurnal Dunia Anak Usia Dini Vol. 1 No. 2 (2019)54-61</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://garuda.kemdiktisaintek.go.id/journal/view/30391</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1 of 1</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>2019</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>10.35473/ijec.v1i2.357</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Sinta 4</t>
         </is>
       </c>
     </row>
@@ -1326,110 +1887,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>judul</t>
+          <t>tahun</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>kategori</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>penulis</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>penerbit</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>tahun</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>kota</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>isbn</t>
+          <t>articles</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Antropobiologi</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>BUKU AJAR</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Swantyka Ilham Prahesti, Nur Intan Rochmawati</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Tiga Cakrawala</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
+      <c r="A2" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
         <v>2022</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Kabupaten Pemalang</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>9786239932343</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Stunting, bagaimana cara penanggulangannya?</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>BUKU MONOGRAF</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Nur Intan Rochmawati, Purbawati, Dewi Fortuna, Muthmainnah, Dian</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>CV. Penerbit Lakeisha</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>2022</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Semarang</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>9786234204384</v>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1443,7 +1985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1454,17 +1996,17 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>leader</t>
+          <t>kategori</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>skema</t>
+          <t>penulis</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>personils</t>
+          <t>penerbit</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1474,58 +2016,79 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>dana</t>
+          <t>kota</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>source</t>
+          <t>isbn</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pengolahan Sampah Plastik melalui Kerajinan Tangan Pendukung Budaya Sehat  desa sidomulyo kecamatan ungaran timur</t>
+          <t>Antropobiologi</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Nur Intan Rochmawati</t>
+          <t>BUKU AJAR</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pengabdian Kepada Masyarakat Kompetitif Nasional ( PKM )</t>
+          <t>Swantyka Ilham Prahesti, Nur Intan Rochmawati</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Personils : Adhi Budi Susilo ; Khifni Kafa Rufaida ;</t>
+          <t>Tiga Cakrawala</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Rp. 31.700.000</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>BIMA SOURCE</t>
-        </is>
+          <t>Kabupaten Pemalang</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>9786239932343</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Stunting, bagaimana cara penanggulangannya?</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BUKU MONOGRAF</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Nur Intan Rochmawati, Purbawati, Dewi Fortuna, Muthmainnah, Dian</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CV. Penerbit Lakeisha</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Semarang</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>9786234204384</v>
       </c>
     </row>
   </sheetData>
@@ -1539,27 +2102,89 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>judul</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>leader</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>skema</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>personils</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>tahun</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>jumlah</t>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>dana</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Pengolahan Sampah Plastik melalui Kerajinan Tangan Pendukung Budaya Sehat  desa sidomulyo kecamatan ungaran timur</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Nur Intan Rochmawati</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Pengabdian Kepada Masyarakat Kompetitif Nasional ( PKM )</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Personils : Adhi Budi Susilo ; Khifni Kafa Rufaida ;</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
         <v>2019</v>
       </c>
-      <c r="B2" t="n">
-        <v>1</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Rp. 31.700.000</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>BIMA SOURCE</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>